<commit_message>
V2: producción 100 % con IA a coste casi cero (pila gratuita, reglas anti contenido no auténtico, escenario financiero)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S9stpomUP8k7EGaEJF9vRy
</commit_message>
<xml_diff>
--- a/docs/youtube/Modelo_YouTube_masivo.xlsx
+++ b/docs/youtube/Modelo_YouTube_masivo.xlsx
@@ -10,8 +10,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conservador" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Optimista" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensibilidad" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Banco 100 ideas" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IA coste casi cero" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensibilidad" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Banco 100 ideas" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4573,289 +4574,1374 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:V43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>Caso</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>Ingresos 12m €</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>Costes 12m €</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>BAI 12m €</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>Caja mínima €</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>YPP</t>
-        </is>
-      </c>
-      <c r="G1" s="2" t="inlineStr">
-        <is>
-          <t>Ingresos mes 12 €</t>
-        </is>
-      </c>
-      <c r="H1" s="2" t="inlineStr">
-        <is>
-          <t>BAI mes 12 €</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Mes</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Vídeos largos</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Shorts</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Vistas vídeos nuevos</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Vistas catálogo</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Vistas largos total</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Vistas Shorts</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Horas públicas 12m</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Suscriptores</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Estado YPP</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Anuncios €</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Afiliación €</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Patrocinio €</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Producto €</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Servicios €</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Ingresos €</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Herramientas €</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Edición y licencias €</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Otros €</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Costes €</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>BAI €</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Caja acumulada €</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Base</t>
+          <t>Nov-26</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1481</v>
+        <v>4</v>
       </c>
       <c r="C2" t="n">
-        <v>10125</v>
+        <v>8</v>
       </c>
       <c r="D2" t="n">
-        <v>-8644</v>
+        <v>3200</v>
       </c>
       <c r="E2" t="n">
-        <v>-8644</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Jul-27</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>3200</v>
       </c>
       <c r="G2" t="n">
-        <v>490</v>
+        <v>6400</v>
       </c>
       <c r="H2" t="n">
-        <v>-780</v>
+        <v>320</v>
+      </c>
+      <c r="I2" t="n">
+        <v>29</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>No elegible</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2">
+        <f>K2+L2+M2+N2+O2</f>
+        <v/>
+      </c>
+      <c r="Q2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T2">
+        <f>Q2+R2+S2</f>
+        <v/>
+      </c>
+      <c r="U2">
+        <f>P2-T2</f>
+        <v/>
+      </c>
+      <c r="V2">
+        <f>U2</f>
+        <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Base con edición propia todo el año (sin externalizar)</t>
+          <t>Dic-26</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1481</v>
+        <v>4</v>
       </c>
       <c r="C3" t="n">
-        <v>3225</v>
+        <v>8</v>
       </c>
       <c r="D3" t="n">
-        <v>-1744</v>
+        <v>4093</v>
       </c>
       <c r="E3" t="n">
-        <v>-1874</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Jul-27</t>
-        </is>
+        <v>800</v>
+      </c>
+      <c r="F3" t="n">
+        <v>4893</v>
       </c>
       <c r="G3" t="n">
-        <v>490</v>
+        <v>9600</v>
       </c>
       <c r="H3" t="n">
-        <v>120</v>
+        <v>809</v>
+      </c>
+      <c r="I3" t="n">
+        <v>73</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>No elegible</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3">
+        <f>K3+L3+M3+N3+O3</f>
+        <v/>
+      </c>
+      <c r="Q3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S3" t="n">
+        <v>0</v>
+      </c>
+      <c r="T3">
+        <f>Q3+R3+S3</f>
+        <v/>
+      </c>
+      <c r="U3">
+        <f>P3-T3</f>
+        <v/>
+      </c>
+      <c r="V3">
+        <f>V2+U3</f>
+        <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Visualizaciones −50 %</t>
+          <t>Ene-27</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>579</v>
+        <v>4</v>
       </c>
       <c r="C4" t="n">
-        <v>10125</v>
+        <v>8</v>
       </c>
       <c r="D4" t="n">
-        <v>-9546</v>
+        <v>5236</v>
       </c>
       <c r="E4" t="n">
-        <v>-9546</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Sep-27</t>
-        </is>
+        <v>1791</v>
+      </c>
+      <c r="F4" t="n">
+        <v>7027</v>
       </c>
       <c r="G4" t="n">
-        <v>245</v>
+        <v>12800</v>
       </c>
       <c r="H4" t="n">
-        <v>-1025</v>
+        <v>1512</v>
+      </c>
+      <c r="I4" t="n">
+        <v>135</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>No elegible</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>2</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4">
+        <f>K4+L4+M4+N4+O4</f>
+        <v/>
+      </c>
+      <c r="Q4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T4">
+        <f>Q4+R4+S4</f>
+        <v/>
+      </c>
+      <c r="U4">
+        <f>P4-T4</f>
+        <v/>
+      </c>
+      <c r="V4">
+        <f>V3+U4</f>
+        <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>RPM a la mitad</t>
+          <t>Feb-27</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1046</v>
+        <v>5</v>
       </c>
       <c r="C5" t="n">
-        <v>10125</v>
+        <v>10</v>
       </c>
       <c r="D5" t="n">
-        <v>-9079</v>
+        <v>8372</v>
       </c>
       <c r="E5" t="n">
-        <v>-9079</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Jul-27</t>
-        </is>
+        <v>3029</v>
+      </c>
+      <c r="F5" t="n">
+        <v>11400</v>
       </c>
       <c r="G5" t="n">
-        <v>336</v>
+        <v>20000</v>
       </c>
       <c r="H5" t="n">
-        <v>-934</v>
+        <v>2652</v>
+      </c>
+      <c r="I5" t="n">
+        <v>237</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>No elegible</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>3</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5">
+        <f>K5+L5+M5+N5+O5</f>
+        <v/>
+      </c>
+      <c r="Q5" t="n">
+        <v>22</v>
+      </c>
+      <c r="R5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T5">
+        <f>Q5+R5+S5</f>
+        <v/>
+      </c>
+      <c r="U5">
+        <f>P5-T5</f>
+        <v/>
+      </c>
+      <c r="V5">
+        <f>V4+U5</f>
+        <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Producción al doble de coste</t>
+          <t>Mar-27</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1481</v>
+        <v>5</v>
       </c>
       <c r="C6" t="n">
-        <v>17970</v>
+        <v>10</v>
       </c>
       <c r="D6" t="n">
-        <v>-16489</v>
+        <v>10709</v>
       </c>
       <c r="E6" t="n">
-        <v>-16489</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Jul-27</t>
-        </is>
+        <v>5000</v>
+      </c>
+      <c r="F6" t="n">
+        <v>15709</v>
       </c>
       <c r="G6" t="n">
-        <v>490</v>
+        <v>25000</v>
       </c>
       <c r="H6" t="n">
-        <v>-1770</v>
+        <v>4223</v>
+      </c>
+      <c r="I6" t="n">
+        <v>375</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>No elegible</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>5</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6">
+        <f>K6+L6+M6+N6+O6</f>
+        <v/>
+      </c>
+      <c r="Q6" t="n">
+        <v>22</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T6">
+        <f>Q6+R6+S6</f>
+        <v/>
+      </c>
+      <c r="U6">
+        <f>P6-T6</f>
+        <v/>
+      </c>
+      <c r="V6">
+        <f>V5+U6</f>
+        <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Monetización YPP 6 meses más tarde</t>
+          <t>Abr-27</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>610</v>
+        <v>5</v>
       </c>
       <c r="C7" t="n">
-        <v>10125</v>
+        <v>10</v>
       </c>
       <c r="D7" t="n">
-        <v>-9515</v>
+        <v>13698</v>
       </c>
       <c r="E7" t="n">
-        <v>-9515</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>no en 12 meses</t>
-        </is>
+        <v>7478</v>
+      </c>
+      <c r="F7" t="n">
+        <v>21175</v>
       </c>
       <c r="G7" t="n">
-        <v>181</v>
+        <v>30000</v>
       </c>
       <c r="H7" t="n">
-        <v>-1089</v>
+        <v>6340</v>
+      </c>
+      <c r="I7" t="n">
+        <v>559</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>No elegible</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>6</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7">
+        <f>K7+L7+M7+N7+O7</f>
+        <v/>
+      </c>
+      <c r="Q7" t="n">
+        <v>22</v>
+      </c>
+      <c r="R7" t="n">
+        <v>0</v>
+      </c>
+      <c r="S7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7">
+        <f>Q7+R7+S7</f>
+        <v/>
+      </c>
+      <c r="U7">
+        <f>P7-T7</f>
+        <v/>
+      </c>
+      <c r="V7">
+        <f>V6+U7</f>
+        <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Un vídeo viral (+1.000.000 vistas en el mes 5)</t>
+          <t>May-27</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>6369</v>
+        <v>6</v>
       </c>
       <c r="C8" t="n">
-        <v>10125</v>
+        <v>12</v>
       </c>
       <c r="D8" t="n">
-        <v>-3756</v>
+        <v>21025</v>
       </c>
       <c r="E8" t="n">
-        <v>-3756</v>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Abr-27</t>
-        </is>
+        <v>10603</v>
+      </c>
+      <c r="F8" t="n">
+        <v>31628</v>
       </c>
       <c r="G8" t="n">
-        <v>1038</v>
+        <v>42000</v>
       </c>
       <c r="H8" t="n">
-        <v>-232</v>
+        <v>9503</v>
+      </c>
+      <c r="I8" t="n">
+        <v>833</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>No elegible</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
+        <v>9</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8">
+        <f>K8+L8+M8+N8+O8</f>
+        <v/>
+      </c>
+      <c r="Q8" t="n">
+        <v>22</v>
+      </c>
+      <c r="R8" t="n">
+        <v>0</v>
+      </c>
+      <c r="S8" t="n">
+        <v>150</v>
+      </c>
+      <c r="T8">
+        <f>Q8+R8+S8</f>
+        <v/>
+      </c>
+      <c r="U8">
+        <f>P8-T8</f>
+        <v/>
+      </c>
+      <c r="V8">
+        <f>V7+U8</f>
+        <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Pérdida de recomendaciones desde el mes 8</t>
+          <t>Jun-27</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>939</v>
+        <v>6</v>
       </c>
       <c r="C9" t="n">
-        <v>10125</v>
+        <v>12</v>
       </c>
       <c r="D9" t="n">
-        <v>-9186</v>
+        <v>26894</v>
       </c>
       <c r="E9" t="n">
-        <v>-9186</v>
-      </c>
-      <c r="F9" t="inlineStr">
+        <v>15435</v>
+      </c>
+      <c r="F9" t="n">
+        <v>42330</v>
+      </c>
+      <c r="G9" t="n">
+        <v>48000</v>
+      </c>
+      <c r="H9" t="n">
+        <v>13736</v>
+      </c>
+      <c r="I9" t="n">
+        <v>1196</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Elegible-revisión</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="n">
+        <v>13</v>
+      </c>
+      <c r="M9" t="n">
+        <v>54</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9">
+        <f>K9+L9+M9+N9+O9</f>
+        <v/>
+      </c>
+      <c r="Q9" t="n">
+        <v>22</v>
+      </c>
+      <c r="R9" t="n">
+        <v>0</v>
+      </c>
+      <c r="S9" t="n">
+        <v>150</v>
+      </c>
+      <c r="T9">
+        <f>Q9+R9+S9</f>
+        <v/>
+      </c>
+      <c r="U9">
+        <f>P9-T9</f>
+        <v/>
+      </c>
+      <c r="V9">
+        <f>V8+U9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>Jul-27</t>
         </is>
       </c>
-      <c r="G9" t="n">
-        <v>301</v>
-      </c>
-      <c r="H9" t="n">
-        <v>-969</v>
+      <c r="B10" t="n">
+        <v>6</v>
+      </c>
+      <c r="C10" t="n">
+        <v>12</v>
+      </c>
+      <c r="D10" t="n">
+        <v>34402</v>
+      </c>
+      <c r="E10" t="n">
+        <v>21541</v>
+      </c>
+      <c r="F10" t="n">
+        <v>55943</v>
+      </c>
+      <c r="G10" t="n">
+        <v>54000</v>
+      </c>
+      <c r="H10" t="n">
+        <v>19331</v>
+      </c>
+      <c r="I10" t="n">
+        <v>1670</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Monetizado</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>140</v>
+      </c>
+      <c r="L10" t="n">
+        <v>17</v>
+      </c>
+      <c r="M10" t="n">
+        <v>69</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10">
+        <f>K10+L10+M10+N10+O10</f>
+        <v/>
+      </c>
+      <c r="Q10" t="n">
+        <v>22</v>
+      </c>
+      <c r="R10" t="n">
+        <v>0</v>
+      </c>
+      <c r="S10" t="n">
+        <v>150</v>
+      </c>
+      <c r="T10">
+        <f>Q10+R10+S10</f>
+        <v/>
+      </c>
+      <c r="U10">
+        <f>P10-T10</f>
+        <v/>
+      </c>
+      <c r="V10">
+        <f>V9+U10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Ago-27</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>6</v>
+      </c>
+      <c r="C11" t="n">
+        <v>12</v>
+      </c>
+      <c r="D11" t="n">
+        <v>44005</v>
+      </c>
+      <c r="E11" t="n">
+        <v>29280</v>
+      </c>
+      <c r="F11" t="n">
+        <v>73285</v>
+      </c>
+      <c r="G11" t="n">
+        <v>60000</v>
+      </c>
+      <c r="H11" t="n">
+        <v>26659</v>
+      </c>
+      <c r="I11" t="n">
+        <v>2287</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Monetizado</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>183</v>
+      </c>
+      <c r="L11" t="n">
+        <v>22</v>
+      </c>
+      <c r="M11" t="n">
+        <v>88</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11">
+        <f>K11+L11+M11+N11+O11</f>
+        <v/>
+      </c>
+      <c r="Q11" t="n">
+        <v>22</v>
+      </c>
+      <c r="R11" t="n">
+        <v>0</v>
+      </c>
+      <c r="S11" t="n">
+        <v>150</v>
+      </c>
+      <c r="T11">
+        <f>Q11+R11+S11</f>
+        <v/>
+      </c>
+      <c r="U11">
+        <f>P11-T11</f>
+        <v/>
+      </c>
+      <c r="V11">
+        <f>V10+U11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Sep-27</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>6</v>
+      </c>
+      <c r="C12" t="n">
+        <v>12</v>
+      </c>
+      <c r="D12" t="n">
+        <v>56288</v>
+      </c>
+      <c r="E12" t="n">
+        <v>39110</v>
+      </c>
+      <c r="F12" t="n">
+        <v>95398</v>
+      </c>
+      <c r="G12" t="n">
+        <v>66000</v>
+      </c>
+      <c r="H12" t="n">
+        <v>36199</v>
+      </c>
+      <c r="I12" t="n">
+        <v>3083</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Monetizado</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
+        <v>238</v>
+      </c>
+      <c r="L12" t="n">
+        <v>29</v>
+      </c>
+      <c r="M12" t="n">
+        <v>113</v>
+      </c>
+      <c r="N12" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12">
+        <f>K12+L12+M12+N12+O12</f>
+        <v/>
+      </c>
+      <c r="Q12" t="n">
+        <v>22</v>
+      </c>
+      <c r="R12" t="n">
+        <v>0</v>
+      </c>
+      <c r="S12" t="n">
+        <v>150</v>
+      </c>
+      <c r="T12">
+        <f>Q12+R12+S12</f>
+        <v/>
+      </c>
+      <c r="U12">
+        <f>P12-T12</f>
+        <v/>
+      </c>
+      <c r="V12">
+        <f>V11+U12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Oct-27</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>6</v>
+      </c>
+      <c r="C13" t="n">
+        <v>12</v>
+      </c>
+      <c r="D13" t="n">
+        <v>72000</v>
+      </c>
+      <c r="E13" t="n">
+        <v>51618</v>
+      </c>
+      <c r="F13" t="n">
+        <v>123618</v>
+      </c>
+      <c r="G13" t="n">
+        <v>72000</v>
+      </c>
+      <c r="H13" t="n">
+        <v>48561</v>
+      </c>
+      <c r="I13" t="n">
+        <v>4108</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Monetizado</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
+        <v>309</v>
+      </c>
+      <c r="L13" t="n">
+        <v>37</v>
+      </c>
+      <c r="M13" t="n">
+        <v>144</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13">
+        <f>K13+L13+M13+N13+O13</f>
+        <v/>
+      </c>
+      <c r="Q13" t="n">
+        <v>22</v>
+      </c>
+      <c r="R13" t="n">
+        <v>0</v>
+      </c>
+      <c r="S13" t="n">
+        <v>150</v>
+      </c>
+      <c r="T13">
+        <f>Q13+R13+S13</f>
+        <v/>
+      </c>
+      <c r="U13">
+        <f>P13-T13</f>
+        <v/>
+      </c>
+      <c r="V13">
+        <f>V12+U13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Hipótesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>nombre</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>IA coste casi cero</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>videos</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>[4, 4, 4, 5, 5, 5, 6, 6, 6, 6, 6, 6]</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>shorts</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>[8, 8, 8, 10, 10, 10, 12, 12, 12, 12, 12, 12]</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>v_inicial</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>800</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>v_final</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>12000</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>cola</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>decaimiento</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>0.96</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>vistas_short</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>[800, 1200, 1600, 2000, 2500, 3000, 3500, 4000, 4500, 5000, 5500, 6000]</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>avd_min</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>6.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>subs_por_mil</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>subs_por_mil_short</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>umbral_horas</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>8000</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>umbral_subs</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>retraso_revision</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>rpm</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>afil_por_mil</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>afil_desde</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>patro_desde</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>patro_cpm</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>patro_por_mes</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>[1, 1, 1, 1, 1, 1, 1, 1, 1, 1, 1, 1]</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>prod_desde</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>prod_conv</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>prod_precio</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>servicios</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>[0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0]</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>herramientas</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>[0, 0, 0, 22, 22, 22, 22, 22, 22, 22, 22, 22]</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>edicion_por_video</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>[0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0]</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>guion_por_video</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>[0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0]</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>otros</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>[0, 0, 0, 0, 0, 0, 150, 150, 150, 150, 150, 150]</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -4869,6 +5955,392 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Caso</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Ingresos 12m €</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Costes 12m €</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>BAI 12m €</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Caja mínima €</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>YPP</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Ingresos mes 12 €</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>BAI mes 12 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1481</v>
+      </c>
+      <c r="C2" t="n">
+        <v>10125</v>
+      </c>
+      <c r="D2" t="n">
+        <v>-8644</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-8644</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Jul-27</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>490</v>
+      </c>
+      <c r="H2" t="n">
+        <v>-780</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Base con edición propia todo el año (sin externalizar)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1481</v>
+      </c>
+      <c r="C3" t="n">
+        <v>3225</v>
+      </c>
+      <c r="D3" t="n">
+        <v>-1744</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-1874</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Jul-27</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>490</v>
+      </c>
+      <c r="H3" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>IA coste casi cero (mismas vistas que la base)</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1481</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1098</v>
+      </c>
+      <c r="D4" t="n">
+        <v>383</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-317</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Jul-27</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>490</v>
+      </c>
+      <c r="H4" t="n">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>IA coste casi cero con −30 % de vistas (voz y estética IA retienen menos)</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>939</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1098</v>
+      </c>
+      <c r="D5" t="n">
+        <v>-159</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-457</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Ago-27</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>343</v>
+      </c>
+      <c r="H5" t="n">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>IA coste casi cero con −60 % de vistas (sin diferenciación)</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>368</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1098</v>
+      </c>
+      <c r="D6" t="n">
+        <v>-730</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-754</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Oct-27</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>196</v>
+      </c>
+      <c r="H6" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Visualizaciones −50 %</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>579</v>
+      </c>
+      <c r="C7" t="n">
+        <v>10125</v>
+      </c>
+      <c r="D7" t="n">
+        <v>-9546</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-9546</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Sep-27</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>245</v>
+      </c>
+      <c r="H7" t="n">
+        <v>-1025</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>RPM a la mitad</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1046</v>
+      </c>
+      <c r="C8" t="n">
+        <v>10125</v>
+      </c>
+      <c r="D8" t="n">
+        <v>-9079</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-9079</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Jul-27</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>336</v>
+      </c>
+      <c r="H8" t="n">
+        <v>-934</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Producción al doble de coste</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1481</v>
+      </c>
+      <c r="C9" t="n">
+        <v>17970</v>
+      </c>
+      <c r="D9" t="n">
+        <v>-16489</v>
+      </c>
+      <c r="E9" t="n">
+        <v>-16489</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Jul-27</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>490</v>
+      </c>
+      <c r="H9" t="n">
+        <v>-1770</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Monetización YPP 6 meses más tarde</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>610</v>
+      </c>
+      <c r="C10" t="n">
+        <v>10125</v>
+      </c>
+      <c r="D10" t="n">
+        <v>-9515</v>
+      </c>
+      <c r="E10" t="n">
+        <v>-9515</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>no en 12 meses</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>181</v>
+      </c>
+      <c r="H10" t="n">
+        <v>-1089</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Un vídeo viral (+1.000.000 vistas en el mes 5)</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>6369</v>
+      </c>
+      <c r="C11" t="n">
+        <v>10125</v>
+      </c>
+      <c r="D11" t="n">
+        <v>-3756</v>
+      </c>
+      <c r="E11" t="n">
+        <v>-3756</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Abr-27</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>1038</v>
+      </c>
+      <c r="H11" t="n">
+        <v>-232</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Pérdida de recomendaciones desde el mes 8</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>939</v>
+      </c>
+      <c r="C12" t="n">
+        <v>10125</v>
+      </c>
+      <c r="D12" t="n">
+        <v>-9186</v>
+      </c>
+      <c r="E12" t="n">
+        <v>-9186</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Jul-27</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>301</v>
+      </c>
+      <c r="H12" t="n">
+        <v>-969</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:S101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>